<commit_message>
Implement 3-tier barcode architecture (Order Unique Code, Product Codes, Book Codes) with scanner verification and live sync
</commit_message>
<xml_diff>
--- a/sample_student_orders.xlsx
+++ b/sample_student_orders.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="49">
   <si>
     <t>Student Name</t>
   </si>
@@ -25,6 +25,12 @@
     <t>Tracking ID</t>
   </si>
   <si>
+    <t>Product Code</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
     <t>Book Code</t>
   </si>
   <si>
@@ -34,88 +40,124 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Rahul Sharma</t>
-  </si>
-  <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>rahul@example.com</t>
-  </si>
-  <si>
-    <t>TR101</t>
-  </si>
-  <si>
-    <t>QB101</t>
-  </si>
-  <si>
-    <t>Quantitative Bank</t>
-  </si>
-  <si>
-    <t>MCQ201</t>
-  </si>
-  <si>
-    <t>MCQ Book</t>
-  </si>
-  <si>
-    <t>Priya Verma</t>
-  </si>
-  <si>
-    <t>9876543211</t>
-  </si>
-  <si>
-    <t>priya@example.com</t>
-  </si>
-  <si>
-    <t>TR102</t>
-  </si>
-  <si>
-    <t>Amit Patel</t>
-  </si>
-  <si>
-    <t>9876543212</t>
-  </si>
-  <si>
-    <t>amit@example.com</t>
-  </si>
-  <si>
-    <t>TR103</t>
-  </si>
-  <si>
-    <t>Sneha Roy</t>
-  </si>
-  <si>
-    <t>9876543213</t>
-  </si>
-  <si>
-    <t>sneha@example.com</t>
-  </si>
-  <si>
-    <t>TR104</t>
-  </si>
-  <si>
-    <t>CS301</t>
-  </si>
-  <si>
-    <t>Computer Science Handbook</t>
-  </si>
-  <si>
-    <t>Vikas Kumar</t>
-  </si>
-  <si>
-    <t>9876543214</t>
-  </si>
-  <si>
-    <t>vikas@example.com</t>
-  </si>
-  <si>
-    <t>TR105</t>
-  </si>
-  <si>
-    <t>ENG401</t>
-  </si>
-  <si>
-    <t>English Comprehension</t>
+    <t>Divya Sharma</t>
+  </si>
+  <si>
+    <t>+919876543210</t>
+  </si>
+  <si>
+    <t>divya.sharma@example.com</t>
+  </si>
+  <si>
+    <t>TRK-IND-9021</t>
+  </si>
+  <si>
+    <t>PRD-FND-01</t>
+  </si>
+  <si>
+    <t>CA Foundation Complete Kit</t>
+  </si>
+  <si>
+    <t>BK-ACC-101</t>
+  </si>
+  <si>
+    <t>Accounting Principles Volume 1</t>
+  </si>
+  <si>
+    <t>BK-LAW-102</t>
+  </si>
+  <si>
+    <t>Business Laws &amp; Corporate Ethics</t>
+  </si>
+  <si>
+    <t>BK-MTH-103</t>
+  </si>
+  <si>
+    <t>Quantitative Aptitude &amp; Logical Reasoning</t>
+  </si>
+  <si>
+    <t>BK-ECO-104</t>
+  </si>
+  <si>
+    <t>Business Economics &amp; Financial Markets</t>
+  </si>
+  <si>
+    <t>Rahul Gupta</t>
+  </si>
+  <si>
+    <t>+919811223344</t>
+  </si>
+  <si>
+    <t>rahul.gupta@example.com</t>
+  </si>
+  <si>
+    <t>TRK-IND-9022</t>
+  </si>
+  <si>
+    <t>PRD-INT-02</t>
+  </si>
+  <si>
+    <t>CA Intermediate Group 1 Combo</t>
+  </si>
+  <si>
+    <t>BK-TAX-201</t>
+  </si>
+  <si>
+    <t>Direct Taxation &amp; GST Practitioner Guide</t>
+  </si>
+  <si>
+    <t>BK-AUD-202</t>
+  </si>
+  <si>
+    <t>Advanced Auditing &amp; Professional Ethics</t>
+  </si>
+  <si>
+    <t>BK-CST-203</t>
+  </si>
+  <si>
+    <t>Cost &amp; Management Accounting Workbook</t>
+  </si>
+  <si>
+    <t>Priya Patel</t>
+  </si>
+  <si>
+    <t>+919988776655</t>
+  </si>
+  <si>
+    <t>priya.patel@example.com</t>
+  </si>
+  <si>
+    <t>TRK-IND-9023</t>
+  </si>
+  <si>
+    <t>PRD-FIN-03</t>
+  </si>
+  <si>
+    <t>CA Final Financial Reporting Kit</t>
+  </si>
+  <si>
+    <t>BK-FRM-301</t>
+  </si>
+  <si>
+    <t>Financial Reporting Masterclass Vol 1</t>
+  </si>
+  <si>
+    <t>BK-SFM-302</t>
+  </si>
+  <si>
+    <t>Strategic Financial Management Practice</t>
+  </si>
+  <si>
+    <t>Aman Verma</t>
+  </si>
+  <si>
+    <t>+919765432109</t>
+  </si>
+  <si>
+    <t>aman.verma@example.com</t>
+  </si>
+  <si>
+    <t>TRK-IND-9024</t>
   </si>
 </sst>
 </file>
@@ -133,9 +175,10 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -145,6 +188,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -160,9 +208,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -502,19 +564,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="36" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,166 +600,330 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" t="s">
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="H11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8">
-        <v>2</v>
+      <c r="I12" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>